<commit_message>
Azimuts en G M S
</commit_message>
<xml_diff>
--- a/09_10_2025/Linea_Tendencia.xlsx
+++ b/09_10_2025/Linea_Tendencia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elkin\Desktop\Vias\DGV\09_10_2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4755BC3-F46C-4DCC-838D-34FEFA4DF24C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BA00D50-3F2A-4519-8584-912D530A9894}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
   <si>
     <t>ESTE</t>
   </si>
@@ -118,14 +118,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -407,462 +407,534 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="C5:H33"/>
+  <dimension ref="C5:I33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="8" width="19" customWidth="1"/>
+    <col min="9" max="9" width="19.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="3:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C5" s="2" t="s">
+    <row r="5" spans="3:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C5" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="2"/>
-      <c r="F5" s="3" t="s">
+      <c r="E5" s="3"/>
+      <c r="F5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="G5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I5" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C6" s="2"/>
+    <row r="6" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C6" s="3"/>
       <c r="D6" s="1" t="s">
         <v>1</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="F6" s="3"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-    </row>
-    <row r="7" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="F6" s="4"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+    </row>
+    <row r="7" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C7" s="1">
         <v>1</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="2">
         <v>1190952.6510000001</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="2">
         <v>838041.85199999996</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
-    </row>
-    <row r="8" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="I7" s="1"/>
+    </row>
+    <row r="8" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
-      <c r="F8" s="4">
+      <c r="F8" s="2">
         <f>((D7-D9)^2+(E7-E9)^2)^(0.5)</f>
         <v>224.37721142095091</v>
       </c>
-      <c r="G8" s="4">
+      <c r="G8" s="2">
         <f>MOD(DEGREES(ATAN2(D9-D7, E9-E7 )), 360)</f>
         <v>160.61255808359681</v>
       </c>
-      <c r="H8" s="1"/>
-    </row>
-    <row r="9" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="H8" s="2" t="str">
+        <f>TEXT(G8/24,"[h]° mm' ss\""")</f>
+        <v>160° 36' 45"</v>
+      </c>
+      <c r="I8" s="1"/>
+    </row>
+    <row r="9" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C9" s="1">
         <v>2</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="2">
         <v>1190740.997</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="2">
         <v>838116.33499999996</v>
       </c>
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
-      <c r="H9" s="4">
-        <f>G10-G8</f>
-        <v>62.284447375024627</v>
-      </c>
-    </row>
-    <row r="10" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="H9" s="1"/>
+      <c r="I9" s="2">
+        <f>G8-G10</f>
+        <v>-62.284447375024627</v>
+      </c>
+    </row>
+    <row r="10" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
-      <c r="F10" s="4">
-        <f t="shared" ref="F9:F32" si="0">((D9-D11)^2+(E9-E11)^2)^(0.5)</f>
+      <c r="F10" s="2">
+        <f t="shared" ref="F10:F32" si="0">((D9-D11)^2+(E9-E11)^2)^(0.5)</f>
         <v>178.76173597548092</v>
       </c>
-      <c r="G10" s="4">
-        <f t="shared" ref="G10:G32" si="1">MOD(DEGREES(ATAN2(D11-D9, E11-E9 )), 360)</f>
+      <c r="G10" s="2">
+        <f t="shared" ref="G10:H10" si="1">MOD(DEGREES(ATAN2(D11-D9, E11-E9 )), 360)</f>
         <v>222.89700545862144</v>
       </c>
-      <c r="H10" s="1"/>
-    </row>
-    <row r="11" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="H10" s="2" t="str">
+        <f t="shared" ref="H10" si="2">TEXT(G10/24,"[h]° mm' ss\""")</f>
+        <v>222° 53' 49"</v>
+      </c>
+      <c r="I10" s="1"/>
+    </row>
+    <row r="11" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C11" s="1">
         <v>3</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="2">
         <v>1190610.04</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="2">
         <v>837994.65500000003</v>
       </c>
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
-      <c r="H11" s="4">
+      <c r="H11" s="1"/>
+      <c r="I11" s="2">
         <f>G12-G10</f>
         <v>-110.42561209368233</v>
       </c>
     </row>
-    <row r="12" spans="3:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
-      <c r="F12" s="4">
+      <c r="F12" s="2">
         <f t="shared" si="0"/>
         <v>171.63842242346485</v>
       </c>
-      <c r="G12" s="4">
-        <f t="shared" ref="G12:G32" si="2">MOD(DEGREES(ATAN2(D13-D11, E13-E11 )), 360)</f>
+      <c r="G12" s="2">
+        <f t="shared" ref="G12:H12" si="3">MOD(DEGREES(ATAN2(D13-D11, E13-E11 )), 360)</f>
         <v>112.4713933649391</v>
       </c>
-      <c r="H12" s="1"/>
-    </row>
-    <row r="13" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="H12" s="2" t="str">
+        <f t="shared" ref="H12" si="4">TEXT(G12/24,"[h]° mm' ss\""")</f>
+        <v>112° 28' 17"</v>
+      </c>
+      <c r="I12" s="1"/>
+    </row>
+    <row r="13" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C13" s="1">
         <v>4</v>
       </c>
-      <c r="D13" s="4">
+      <c r="D13" s="2">
         <v>1190544.436</v>
       </c>
-      <c r="E13" s="4">
+      <c r="E13" s="2">
         <v>838153.26100000006</v>
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
-      <c r="H13" s="4">
-        <f t="shared" ref="H13:H31" si="3">G14-G12</f>
+      <c r="H13" s="1"/>
+      <c r="I13" s="2">
+        <f>G14-G12</f>
         <v>83.617297423928903</v>
       </c>
     </row>
-    <row r="14" spans="3:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
-      <c r="F14" s="4">
+      <c r="F14" s="2">
         <f t="shared" si="0"/>
         <v>218.15425743277078</v>
       </c>
-      <c r="G14" s="4">
-        <f t="shared" ref="G14:G32" si="4">MOD(DEGREES(ATAN2(D15-D13, E15-E13 )), 360)</f>
+      <c r="G14" s="2">
+        <f t="shared" ref="G14:H14" si="5">MOD(DEGREES(ATAN2(D15-D13, E15-E13 )), 360)</f>
         <v>196.08869078886801</v>
       </c>
-      <c r="H14" s="1"/>
-    </row>
-    <row r="15" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="H14" s="2" t="str">
+        <f t="shared" ref="H14" si="6">TEXT(G14/24,"[h]° mm' ss\""")</f>
+        <v>196° 05' 19"</v>
+      </c>
+      <c r="I14" s="1"/>
+    </row>
+    <row r="15" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C15" s="1">
         <v>5</v>
       </c>
-      <c r="D15" s="4">
+      <c r="D15" s="2">
         <v>1190334.8259999999</v>
       </c>
-      <c r="E15" s="4">
+      <c r="E15" s="2">
         <v>838092.80500000005</v>
       </c>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
-      <c r="H15" s="4">
-        <f t="shared" ref="H15:H31" si="5">G16-G14</f>
+      <c r="H15" s="1"/>
+      <c r="I15" s="2">
+        <f>G16-G14</f>
         <v>-13.965241132994464</v>
       </c>
     </row>
-    <row r="16" spans="3:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
-      <c r="F16" s="4">
+      <c r="F16" s="2">
         <f t="shared" si="0"/>
         <v>277.55059044421034</v>
       </c>
-      <c r="G16" s="4">
-        <f t="shared" ref="G16:G32" si="6">MOD(DEGREES(ATAN2(D17-D15, E17-E15 )), 360)</f>
+      <c r="G16" s="2">
+        <f t="shared" ref="G16:H16" si="7">MOD(DEGREES(ATAN2(D17-D15, E17-E15 )), 360)</f>
         <v>182.12344965587354</v>
       </c>
-      <c r="H16" s="1"/>
-    </row>
-    <row r="17" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="H16" s="2" t="str">
+        <f t="shared" ref="H16" si="8">TEXT(G16/24,"[h]° mm' ss\""")</f>
+        <v>182° 07' 24"</v>
+      </c>
+      <c r="I16" s="1"/>
+    </row>
+    <row r="17" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C17" s="1">
         <v>6</v>
       </c>
-      <c r="D17" s="4">
+      <c r="D17" s="2">
         <v>1190057.466</v>
       </c>
-      <c r="E17" s="4">
+      <c r="E17" s="2">
         <v>838082.52099999995</v>
       </c>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
-      <c r="H17" s="4">
-        <f t="shared" ref="H17:H31" si="7">G18-G16</f>
+      <c r="H17" s="1"/>
+      <c r="I17" s="2">
+        <f>G18-G16</f>
         <v>122.99455713695593</v>
       </c>
     </row>
-    <row r="18" spans="3:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
-      <c r="F18" s="4">
+      <c r="F18" s="2">
         <f t="shared" si="0"/>
         <v>183.34069665514104</v>
       </c>
-      <c r="G18" s="4">
-        <f t="shared" ref="G18:G32" si="8">MOD(DEGREES(ATAN2(D19-D17, E19-E17 )), 360)</f>
+      <c r="G18" s="2">
+        <f t="shared" ref="G18:H18" si="9">MOD(DEGREES(ATAN2(D19-D17, E19-E17 )), 360)</f>
         <v>305.11800679282948</v>
       </c>
-      <c r="H18" s="1"/>
-    </row>
-    <row r="19" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="H18" s="2" t="str">
+        <f t="shared" ref="H18" si="10">TEXT(G18/24,"[h]° mm' ss\""")</f>
+        <v>305° 07' 05"</v>
+      </c>
+      <c r="I18" s="1"/>
+    </row>
+    <row r="19" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C19" s="1">
         <v>7</v>
       </c>
-      <c r="D19" s="4">
+      <c r="D19" s="2">
         <v>1190162.9350000001</v>
       </c>
-      <c r="E19" s="4">
+      <c r="E19" s="2">
         <v>837932.554</v>
       </c>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
-      <c r="H19" s="4">
-        <f t="shared" ref="H19:H31" si="9">G20-G18</f>
+      <c r="H19" s="1"/>
+      <c r="I19" s="2">
+        <f>G20-G18</f>
         <v>-8.9685807828532802</v>
       </c>
     </row>
-    <row r="20" spans="3:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
-      <c r="F20" s="4">
+      <c r="F20" s="2">
         <f t="shared" si="0"/>
         <v>175.82844003179724</v>
       </c>
-      <c r="G20" s="4">
-        <f t="shared" ref="G20:G32" si="10">MOD(DEGREES(ATAN2(D21-D19, E21-E19 )), 360)</f>
+      <c r="G20" s="2">
+        <f t="shared" ref="G20:H20" si="11">MOD(DEGREES(ATAN2(D21-D19, E21-E19 )), 360)</f>
         <v>296.1494260099762</v>
       </c>
-      <c r="H20" s="1"/>
-    </row>
-    <row r="21" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="H20" s="2" t="str">
+        <f t="shared" ref="H20" si="12">TEXT(G20/24,"[h]° mm' ss\""")</f>
+        <v>296° 08' 58"</v>
+      </c>
+      <c r="I20" s="1"/>
+    </row>
+    <row r="21" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C21" s="1">
         <v>8</v>
       </c>
-      <c r="D21" s="4">
+      <c r="D21" s="2">
         <v>1190240.425</v>
       </c>
-      <c r="E21" s="4">
+      <c r="E21" s="2">
         <v>837774.72199999995</v>
       </c>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
-      <c r="H21" s="4">
-        <f t="shared" ref="H21:H31" si="11">G22-G20</f>
+      <c r="H21" s="1"/>
+      <c r="I21" s="2">
+        <f>G22-G20</f>
         <v>-57.810371372826637</v>
       </c>
     </row>
-    <row r="22" spans="3:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
-      <c r="F22" s="4">
+      <c r="F22" s="2">
         <f t="shared" si="0"/>
         <v>175.72771585608109</v>
       </c>
-      <c r="G22" s="4">
-        <f t="shared" ref="G22:G32" si="12">MOD(DEGREES(ATAN2(D23-D21, E23-E21 )), 360)</f>
+      <c r="G22" s="2">
+        <f t="shared" ref="G22:H22" si="13">MOD(DEGREES(ATAN2(D23-D21, E23-E21 )), 360)</f>
         <v>238.33905463714956</v>
       </c>
-      <c r="H22" s="1"/>
-    </row>
-    <row r="23" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="H22" s="2" t="str">
+        <f t="shared" ref="H22" si="14">TEXT(G22/24,"[h]° mm' ss\""")</f>
+        <v>238° 20' 21"</v>
+      </c>
+      <c r="I22" s="1"/>
+    </row>
+    <row r="23" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C23" s="1">
         <v>9</v>
       </c>
-      <c r="D23" s="4">
+      <c r="D23" s="2">
         <v>1190148.1869999999</v>
       </c>
-      <c r="E23" s="4">
+      <c r="E23" s="2">
         <v>837625.14800000004</v>
       </c>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
-      <c r="H23" s="4">
-        <f t="shared" ref="H23:H31" si="13">G24-G22</f>
+      <c r="H23" s="1"/>
+      <c r="I23" s="2">
+        <f>G24-G22</f>
         <v>-92.81713441913783</v>
       </c>
     </row>
-    <row r="24" spans="3:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
-      <c r="F24" s="4">
+      <c r="F24" s="2">
         <f t="shared" si="0"/>
         <v>211.40597689272116</v>
       </c>
-      <c r="G24" s="4">
-        <f t="shared" ref="G24:G32" si="14">MOD(DEGREES(ATAN2(D25-D23, E25-E23 )), 360)</f>
+      <c r="G24" s="2">
+        <f t="shared" ref="G24:H24" si="15">MOD(DEGREES(ATAN2(D25-D23, E25-E23 )), 360)</f>
         <v>145.52192021801173</v>
       </c>
-      <c r="H24" s="1"/>
-    </row>
-    <row r="25" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="H24" s="2" t="str">
+        <f t="shared" ref="H24" si="16">TEXT(G24/24,"[h]° mm' ss\""")</f>
+        <v>145° 31' 19"</v>
+      </c>
+      <c r="I24" s="1"/>
+    </row>
+    <row r="25" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C25" s="1">
         <v>10</v>
       </c>
-      <c r="D25" s="4">
+      <c r="D25" s="2">
         <v>1189973.916</v>
       </c>
-      <c r="E25" s="4">
+      <c r="E25" s="2">
         <v>837744.82299999997</v>
       </c>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
-      <c r="H25" s="4">
-        <f t="shared" ref="H25:H31" si="15">G26-G24</f>
+      <c r="H25" s="1"/>
+      <c r="I25" s="2">
+        <f>G26-G24</f>
         <v>62.548972017699867</v>
       </c>
     </row>
-    <row r="26" spans="3:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
-      <c r="F26" s="4">
+      <c r="F26" s="2">
         <f t="shared" si="0"/>
         <v>166.96358829980309</v>
       </c>
-      <c r="G26" s="4">
-        <f t="shared" ref="G26:G32" si="16">MOD(DEGREES(ATAN2(D27-D25, E27-E25 )), 360)</f>
+      <c r="G26" s="2">
+        <f t="shared" ref="G26:H26" si="17">MOD(DEGREES(ATAN2(D27-D25, E27-E25 )), 360)</f>
         <v>208.0708922357116</v>
       </c>
-      <c r="H26" s="1"/>
-    </row>
-    <row r="27" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="H26" s="2" t="str">
+        <f t="shared" ref="H26" si="18">TEXT(G26/24,"[h]° mm' ss\""")</f>
+        <v>208° 04' 15"</v>
+      </c>
+      <c r="I26" s="1"/>
+    </row>
+    <row r="27" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C27" s="1">
         <v>11</v>
       </c>
-      <c r="D27" s="4">
+      <c r="D27" s="2">
         <v>1189826.5930000001</v>
       </c>
-      <c r="E27" s="4">
+      <c r="E27" s="2">
         <v>837666.25600000005</v>
       </c>
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
-      <c r="H27" s="4">
-        <f t="shared" ref="H27:H31" si="17">G28-G26</f>
+      <c r="H27" s="1"/>
+      <c r="I27" s="2">
+        <f>G28-G26</f>
         <v>-73.442873112404754</v>
       </c>
     </row>
-    <row r="28" spans="3:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
-      <c r="F28" s="4">
+      <c r="F28" s="2">
         <f t="shared" si="0"/>
         <v>179.71073317431959</v>
       </c>
-      <c r="G28" s="4">
-        <f t="shared" ref="G28:G32" si="18">MOD(DEGREES(ATAN2(D29-D27, E29-E27 )), 360)</f>
+      <c r="G28" s="2">
+        <f t="shared" ref="G28:H28" si="19">MOD(DEGREES(ATAN2(D29-D27, E29-E27 )), 360)</f>
         <v>134.62801912330684</v>
       </c>
-      <c r="H28" s="1"/>
-    </row>
-    <row r="29" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="H28" s="2" t="str">
+        <f t="shared" ref="H28" si="20">TEXT(G28/24,"[h]° mm' ss\""")</f>
+        <v>134° 37' 41"</v>
+      </c>
+      <c r="I28" s="1"/>
+    </row>
+    <row r="29" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C29" s="1">
         <v>12</v>
       </c>
-      <c r="D29" s="4">
+      <c r="D29" s="2">
         <v>1189700.3459999999</v>
       </c>
-      <c r="E29" s="4">
+      <c r="E29" s="2">
         <v>837794.15300000005</v>
       </c>
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
-      <c r="H29" s="4">
-        <f t="shared" ref="H29:H31" si="19">G30-G28</f>
+      <c r="H29" s="1"/>
+      <c r="I29" s="2">
+        <f>G30-G28</f>
         <v>71.239044665836531</v>
       </c>
     </row>
-    <row r="30" spans="3:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
-      <c r="F30" s="4">
+      <c r="F30" s="2">
         <f t="shared" si="0"/>
         <v>183.41009109917889</v>
       </c>
-      <c r="G30" s="4">
-        <f t="shared" ref="G30:G32" si="20">MOD(DEGREES(ATAN2(D31-D29, E31-E29 )), 360)</f>
+      <c r="G30" s="2">
+        <f t="shared" ref="G30:H30" si="21">MOD(DEGREES(ATAN2(D31-D29, E31-E29 )), 360)</f>
         <v>205.86706378914337</v>
       </c>
-      <c r="H30" s="1"/>
-    </row>
-    <row r="31" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="H30" s="2" t="str">
+        <f t="shared" ref="H30" si="22">TEXT(G30/24,"[h]° mm' ss\""")</f>
+        <v>205° 52' 01"</v>
+      </c>
+      <c r="I30" s="1"/>
+    </row>
+    <row r="31" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C31" s="1">
         <v>13</v>
       </c>
-      <c r="D31" s="4">
+      <c r="D31" s="2">
         <v>1189535.3119999999</v>
       </c>
-      <c r="E31" s="4">
+      <c r="E31" s="2">
         <v>837714.13399999996</v>
       </c>
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
-      <c r="H31" s="4">
-        <f t="shared" ref="H31" si="21">G32-G30</f>
+      <c r="H31" s="1"/>
+      <c r="I31" s="2">
+        <f>G32-G30</f>
         <v>-28.546823644955253</v>
       </c>
     </row>
-    <row r="32" spans="3:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
-      <c r="F32" s="4">
+      <c r="F32" s="2">
         <f t="shared" si="0"/>
         <v>200.21994986008028</v>
       </c>
-      <c r="G32" s="4">
-        <f t="shared" ref="G32" si="22">MOD(DEGREES(ATAN2(D33-D31, E33-E31 )), 360)</f>
+      <c r="G32" s="2">
+        <f t="shared" ref="G32:H32" si="23">MOD(DEGREES(ATAN2(D33-D31, E33-E31 )), 360)</f>
         <v>177.32024014418812</v>
       </c>
-      <c r="H32" s="1"/>
-    </row>
-    <row r="33" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="H32" s="2" t="str">
+        <f t="shared" ref="H32" si="24">TEXT(G32/24,"[h]° mm' ss\""")</f>
+        <v>177° 19' 13"</v>
+      </c>
+      <c r="I32" s="1"/>
+    </row>
+    <row r="33" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C33" s="1">
         <v>14</v>
       </c>
-      <c r="D33" s="4">
+      <c r="D33" s="2">
         <v>1189335.311</v>
       </c>
-      <c r="E33" s="4">
+      <c r="E33" s="2">
         <v>837723.495</v>
       </c>
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
-      <c r="H33" s="4"/>
+      <c r="H33" s="1"/>
+      <c r="I33" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="D5:E5"/>
     <mergeCell ref="C5:C6"/>
     <mergeCell ref="F5:F6"/>
     <mergeCell ref="G5:G6"/>
+    <mergeCell ref="I5:I6"/>
     <mergeCell ref="H5:H6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>